<commit_message>
fix(ai-skill-studio): repair quote formula and print area
</commit_message>
<xml_diff>
--- a/docs/commercial/business-32-ai-skill-studio/customer-package/Business32_Pilot_Quote_Template.xlsx
+++ b/docs/commercial/business-32-ai-skill-studio/customer-package/Business32_Pilot_Quote_Template.xlsx
@@ -16,7 +16,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="견적" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="가정·제외사항" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm.Print_Area" localSheetId="6">'견적'!$A$1:$C$9</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -1352,6 +1354,9 @@
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="44" customWidth="1" min="3" max="3"/>
+    <col hidden="1" width="13" customWidth="1" min="7" max="7"/>
+    <col hidden="1" width="13" customWidth="1" min="8" max="8"/>
+    <col hidden="1" width="13" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1493,11 +1498,11 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>계약 자동 확정 없음</t>
+          <t>가격 범위 판정</t>
         </is>
       </c>
       <c r="B9" s="4">
-        <f>IF(AND(B4&gt;=VLOOKUP(Offer!$B$4,$G$4:$I$6,2,FALSE),B4&lt;=VLOOKUP(Offer!$B$4,$G$4:$I$6,3,FALSE)),"가설 범위 내","⚠ 범위 밖 가격 — 가설 범위를 확인하세요")</f>
+        <f>IF(AND(B4&gt;=VLOOKUP('Offer 선택'!$B$4,$G$4:$I$6,2,FALSE),B4&lt;=VLOOKUP('Offer 선택'!$B$4,$G$4:$I$6,3,FALSE)),"가설 범위 내","⚠ 범위 밖 가격 — 가설 범위를 확인하세요")</f>
         <v/>
       </c>
       <c r="C9" t="inlineStr">

</xml_diff>